<commit_message>
Solving Task 2 - SQL
</commit_message>
<xml_diff>
--- a/02_spreadsheet/spreadsheet_workbook.xlsx
+++ b/02_spreadsheet/spreadsheet_workbook.xlsx
@@ -1914,7 +1914,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" ht="15.75" hidden="1" customHeight="1">
+    <row r="2" ht="15.75" customHeight="1">
       <c r="A2" s="1" t="s">
         <v>19</v>
       </c>
@@ -1982,7 +1982,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" ht="15.75" hidden="1" customHeight="1">
+    <row r="3" ht="15.75" customHeight="1">
       <c r="A3" s="1" t="s">
         <v>27</v>
       </c>
@@ -2183,7 +2183,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" ht="15.75" hidden="1" customHeight="1">
+    <row r="6" ht="15.75" customHeight="1">
       <c r="A6" s="1" t="s">
         <v>42</v>
       </c>
@@ -2313,7 +2313,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" ht="15.75" hidden="1" customHeight="1">
+    <row r="8" ht="15.75" customHeight="1">
       <c r="A8" s="1" t="s">
         <v>48</v>
       </c>
@@ -2446,7 +2446,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" ht="15.75" hidden="1" customHeight="1">
+    <row r="10" ht="15.75" customHeight="1">
       <c r="A10" s="1" t="s">
         <v>55</v>
       </c>
@@ -2579,7 +2579,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="12" ht="15.75" hidden="1" customHeight="1">
+    <row r="12" ht="15.75" customHeight="1">
       <c r="A12" s="1" t="s">
         <v>59</v>
       </c>
@@ -2709,7 +2709,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="15.75" hidden="1" customHeight="1">
+    <row r="14" ht="15.75" customHeight="1">
       <c r="A14" s="1" t="s">
         <v>65</v>
       </c>
@@ -2845,7 +2845,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="16" ht="15.75" hidden="1" customHeight="1">
+    <row r="16" ht="15.75" customHeight="1">
       <c r="A16" s="1" t="s">
         <v>70</v>
       </c>
@@ -3111,7 +3111,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" ht="15.75" hidden="1" customHeight="1">
+    <row r="20" ht="15.75" customHeight="1">
       <c r="A20" s="1" t="s">
         <v>80</v>
       </c>
@@ -3179,7 +3179,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="21" ht="15.75" hidden="1" customHeight="1">
+    <row r="21" ht="15.75" customHeight="1">
       <c r="A21" s="1" t="s">
         <v>82</v>
       </c>
@@ -3312,7 +3312,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="23" ht="15.75" hidden="1" customHeight="1">
+    <row r="23" ht="15.75" customHeight="1">
       <c r="A23" s="1" t="s">
         <v>86</v>
       </c>
@@ -3380,7 +3380,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="24" ht="15.75" hidden="1" customHeight="1">
+    <row r="24" ht="15.75" customHeight="1">
       <c r="A24" s="1" t="s">
         <v>87</v>
       </c>
@@ -3516,7 +3516,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="26" ht="15.75" hidden="1" customHeight="1">
+    <row r="26" ht="15.75" customHeight="1">
       <c r="A26" s="1" t="s">
         <v>94</v>
       </c>
@@ -3652,7 +3652,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="28" ht="15.75" hidden="1" customHeight="1">
+    <row r="28" ht="15.75" customHeight="1">
       <c r="A28" s="1" t="s">
         <v>97</v>
       </c>
@@ -3720,7 +3720,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="29" ht="15.75" hidden="1" customHeight="1">
+    <row r="29" ht="15.75" customHeight="1">
       <c r="A29" s="1" t="s">
         <v>101</v>
       </c>
@@ -3788,7 +3788,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="30" ht="15.75" hidden="1" customHeight="1">
+    <row r="30" ht="15.75" customHeight="1">
       <c r="A30" s="1" t="s">
         <v>105</v>
       </c>
@@ -3856,7 +3856,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="31" ht="15.75" hidden="1" customHeight="1">
+    <row r="31" ht="15.75" customHeight="1">
       <c r="A31" s="1" t="s">
         <v>108</v>
       </c>
@@ -4903,14 +4903,7 @@
     <row r="999" ht="15.75" customHeight="1"/>
     <row r="1000" ht="15.75" customHeight="1"/>
   </sheetData>
-  <autoFilter ref="$A$1:$AG$32">
-    <filterColumn colId="4">
-      <filters blank="1">
-        <filter val="Beta Stores"/>
-        <filter val="Eco Home"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="$A$1:$AG$32"/>
   <drawing r:id="rId1"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Adding dashboard link file
</commit_message>
<xml_diff>
--- a/02_spreadsheet/spreadsheet_workbook.xlsx
+++ b/02_spreadsheet/spreadsheet_workbook.xlsx
@@ -713,12 +713,12 @@
     </cacheField>
     <cacheField name="transaction_date_cleaned" numFmtId="0">
       <sharedItems>
-        <s v="2026_03-01"/>
-        <s v="2026_03-02"/>
-        <s v="2026_03-03"/>
-        <s v="2026_03-04"/>
-        <s v="2026_03-05"/>
-        <s v="2026_03-06"/>
+        <s v="2026-03-01"/>
+        <s v="2026-03-02"/>
+        <s v="2026-03-03"/>
+        <s v="2026-03-04"/>
+        <s v="2026-03-05"/>
+        <s v="2026-03-06"/>
       </sharedItems>
     </cacheField>
     <cacheField name="merchant_name" numFmtId="0">
@@ -1922,8 +1922,8 @@
         <v>46082.0</v>
       </c>
       <c r="C2" s="1" t="str">
-        <f t="shared" ref="C2:C31" si="1">TEXT(if(or(B2="", B2="UNKNOWN", B2="ERROR"), "1900-01-01", B2), "YYYY_MM-DD")</f>
-        <v>2026_03-01</v>
+        <f t="shared" ref="C2:C31" si="1">TEXT(if(or(B2="", B2="UNKNOWN", B2="ERROR"), "1900-01-01", B2), "YYYY-MM-DD")</f>
+        <v>2026-03-01</v>
       </c>
       <c r="D2" s="1" t="s">
         <v>20</v>
@@ -1991,7 +1991,7 @@
       </c>
       <c r="C3" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-01</v>
+        <v>2026-03-01</v>
       </c>
       <c r="D3" s="1" t="s">
         <v>28</v>
@@ -2056,7 +2056,7 @@
       </c>
       <c r="C4" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-01</v>
+        <v>2026-03-01</v>
       </c>
       <c r="D4" s="1" t="s">
         <v>33</v>
@@ -2124,7 +2124,7 @@
       </c>
       <c r="C5" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-02</v>
+        <v>2026-03-02</v>
       </c>
       <c r="D5" s="1" t="s">
         <v>38</v>
@@ -2192,7 +2192,7 @@
       </c>
       <c r="C6" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-02</v>
+        <v>2026-03-02</v>
       </c>
       <c r="D6" s="1" t="s">
         <v>43</v>
@@ -2257,7 +2257,7 @@
       </c>
       <c r="C7" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-02</v>
+        <v>2026-03-02</v>
       </c>
       <c r="D7" s="1" t="s">
         <v>38</v>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="C8" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-02</v>
+        <v>2026-03-02</v>
       </c>
       <c r="D8" s="1" t="s">
         <v>49</v>
@@ -2390,7 +2390,7 @@
       </c>
       <c r="C9" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-03</v>
+        <v>2026-03-03</v>
       </c>
       <c r="D9" s="1" t="s">
         <v>33</v>
@@ -2455,7 +2455,7 @@
       </c>
       <c r="C10" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-03</v>
+        <v>2026-03-03</v>
       </c>
       <c r="D10" s="1" t="s">
         <v>43</v>
@@ -2523,7 +2523,7 @@
       </c>
       <c r="C11" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-03</v>
+        <v>2026-03-03</v>
       </c>
       <c r="D11" s="1" t="s">
         <v>57</v>
@@ -2588,7 +2588,7 @@
       </c>
       <c r="C12" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-03</v>
+        <v>2026-03-03</v>
       </c>
       <c r="D12" s="1" t="s">
         <v>49</v>
@@ -2650,7 +2650,7 @@
       </c>
       <c r="C13" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-04</v>
+        <v>2026-03-04</v>
       </c>
       <c r="D13" s="1" t="s">
         <v>38</v>
@@ -2718,7 +2718,7 @@
       </c>
       <c r="C14" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-04</v>
+        <v>2026-03-04</v>
       </c>
       <c r="D14" s="1" t="s">
         <v>20</v>
@@ -2786,7 +2786,7 @@
       </c>
       <c r="C15" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-04</v>
+        <v>2026-03-04</v>
       </c>
       <c r="D15" s="1" t="s">
         <v>38</v>
@@ -2854,7 +2854,7 @@
       </c>
       <c r="C16" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-04</v>
+        <v>2026-03-04</v>
       </c>
       <c r="D16" s="1" t="s">
         <v>43</v>
@@ -2919,7 +2919,7 @@
       </c>
       <c r="C17" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-05</v>
+        <v>2026-03-05</v>
       </c>
       <c r="D17" s="1" t="s">
         <v>38</v>
@@ -2984,7 +2984,7 @@
       </c>
       <c r="C18" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-05</v>
+        <v>2026-03-05</v>
       </c>
       <c r="D18" s="1" t="s">
         <v>38</v>
@@ -3052,7 +3052,7 @@
       </c>
       <c r="C19" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-05</v>
+        <v>2026-03-05</v>
       </c>
       <c r="D19" s="1" t="s">
         <v>33</v>
@@ -3120,7 +3120,7 @@
       </c>
       <c r="C20" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-05</v>
+        <v>2026-03-05</v>
       </c>
       <c r="D20" s="1" t="s">
         <v>49</v>
@@ -3188,7 +3188,7 @@
       </c>
       <c r="C21" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-05</v>
+        <v>2026-03-05</v>
       </c>
       <c r="D21" s="1" t="s">
         <v>43</v>
@@ -3256,7 +3256,7 @@
       </c>
       <c r="C22" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-06</v>
+        <v>2026-03-06</v>
       </c>
       <c r="D22" s="1" t="s">
         <v>84</v>
@@ -3321,7 +3321,7 @@
       </c>
       <c r="C23" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-06</v>
+        <v>2026-03-06</v>
       </c>
       <c r="D23" s="1" t="s">
         <v>28</v>
@@ -3389,7 +3389,7 @@
       </c>
       <c r="C24" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-01</v>
+        <v>2026-03-01</v>
       </c>
       <c r="D24" s="1" t="s">
         <v>88</v>
@@ -3457,7 +3457,7 @@
       </c>
       <c r="C25" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-02</v>
+        <v>2026-03-02</v>
       </c>
       <c r="D25" s="1" t="s">
         <v>92</v>
@@ -3525,7 +3525,7 @@
       </c>
       <c r="C26" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-03</v>
+        <v>2026-03-03</v>
       </c>
       <c r="D26" s="1" t="s">
         <v>88</v>
@@ -3593,7 +3593,7 @@
       </c>
       <c r="C27" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-05</v>
+        <v>2026-03-05</v>
       </c>
       <c r="D27" s="1" t="s">
         <v>92</v>
@@ -3661,7 +3661,7 @@
       </c>
       <c r="C28" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-01</v>
+        <v>2026-03-01</v>
       </c>
       <c r="D28" s="1" t="s">
         <v>98</v>
@@ -3729,7 +3729,7 @@
       </c>
       <c r="C29" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-02</v>
+        <v>2026-03-02</v>
       </c>
       <c r="D29" s="1" t="s">
         <v>102</v>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="C30" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-04</v>
+        <v>2026-03-04</v>
       </c>
       <c r="D30" s="1" t="s">
         <v>106</v>
@@ -3865,7 +3865,7 @@
       </c>
       <c r="C31" s="1" t="str">
         <f t="shared" si="1"/>
-        <v>2026_03-06</v>
+        <v>2026-03-06</v>
       </c>
       <c r="D31" s="1" t="s">
         <v>98</v>

</xml_diff>